<commit_message>
Exercise 3.3, upload files
</commit_message>
<xml_diff>
--- a/src/activities/RA2/lesson_03/data/KIPs-area-gestion-hospitalaria.xlsx
+++ b/src/activities/RA2/lesson_03/data/KIPs-area-gestion-hospitalaria.xlsx
@@ -8,19 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Debian\home\dcueli\projects\courses\regulated\ai-and-big-data\p1\bigdata_sys\src\activities\RA2\lesson_03\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D0D0205-5E05-4E3B-B4DA-BBB319FBB253}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FDA2904-6E6D-46BC-907F-A41F5FF25219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{E2C55299-9E87-4FEC-B842-C06A78B44C56}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{E2C55299-9E87-4FEC-B842-C06A78B44C56}"/>
   </bookViews>
   <sheets>
-    <sheet name="KIPs simple" sheetId="1" r:id="rId1"/>
-    <sheet name="Hoja1" sheetId="2" r:id="rId2"/>
-    <sheet name="Hoja2" sheetId="3" r:id="rId3"/>
+    <sheet name="INCLASNS KPIS" sheetId="3" r:id="rId1"/>
+    <sheet name="Simple List KIPs" sheetId="1" r:id="rId2"/>
+    <sheet name="General KPIs" sheetId="2" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Hoja1!$A$7:$E$84</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Hoja2!$B$19:$K$48</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'KIPs simple'!$A$1:$E$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'General KPIs'!$A$9:$E$86</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'INCLASNS KPIS'!$B$19:$K$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Simple List KIPs'!$A$1:$E$12</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="305">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="307">
   <si>
     <t>Área de Gestión</t>
   </si>
@@ -1062,12 +1062,18 @@
   <si>
     <t>KPI:ID</t>
   </si>
+  <si>
+    <t xml:space="preserve">* Propuesta general de gestión hospitalaria, no verificada de indicadores oficiales del Sistema Nacional de Salud (SNS). </t>
+  </si>
+  <si>
+    <t>(1–5) Estimación orientativa de cuánto se utiliza normalmente el indicador en la gestión hospitalaria, es decir la frecuencia con la que las supervisiones del hospital monitorizan el dato</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1127,6 +1133,15 @@
       <color theme="1"/>
       <name val="Consolas"/>
       <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <color theme="5" tint="-0.499984740745262"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="10">
@@ -1495,7 +1510,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1535,13 +1550,24 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Entrada" xfId="2" builtinId="20"/>
     <cellStyle name="Neutral" xfId="1" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFF00"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
@@ -1879,1628 +1905,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8B34BCC-6511-4EA4-B349-2A5DFD03ED2A}">
-  <dimension ref="A1:E18"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="35" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="8"/>
-      <c r="B13" s="9"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="10"/>
-    </row>
-    <row r="18" spans="3:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C18" s="1"/>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:E12" xr:uid="{C8B34BCC-6511-4EA4-B349-2A5DFD03ED2A}"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9A493EE-0271-4CD7-8525-04393AE8438C}">
-  <dimension ref="A1:E84"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="40.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="37.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="45" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.5703125" customWidth="1"/>
-    <col min="5" max="5" width="14.140625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
-        <v>205</v>
-      </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="15"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
-        <v>191</v>
-      </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="17"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="18" t="s">
-        <v>204</v>
-      </c>
-      <c r="B3" s="11"/>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="17"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="16" t="s">
-        <v>36</v>
-      </c>
-      <c r="B4" s="11"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="17"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="19" t="s">
-        <v>203</v>
-      </c>
-      <c r="B5" s="20"/>
-      <c r="C5" s="20"/>
-      <c r="D5" s="20"/>
-      <c r="E5" s="21"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="22" t="s">
-        <v>191</v>
-      </c>
-      <c r="B7" s="23" t="s">
-        <v>1</v>
-      </c>
-      <c r="C7" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="D7" s="23" t="s">
-        <v>36</v>
-      </c>
-      <c r="E7" s="24" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>192</v>
-      </c>
-      <c r="B8" t="s">
-        <v>38</v>
-      </c>
-      <c r="C8" t="s">
-        <v>39</v>
-      </c>
-      <c r="D8">
-        <v>4</v>
-      </c>
-      <c r="E8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>192</v>
-      </c>
-      <c r="B9" t="s">
-        <v>40</v>
-      </c>
-      <c r="C9" t="s">
-        <v>41</v>
-      </c>
-      <c r="D9">
-        <v>5</v>
-      </c>
-      <c r="E9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>192</v>
-      </c>
-      <c r="B10" t="s">
-        <v>42</v>
-      </c>
-      <c r="C10" t="s">
-        <v>43</v>
-      </c>
-      <c r="D10">
-        <v>5</v>
-      </c>
-      <c r="E10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>192</v>
-      </c>
-      <c r="B11" t="s">
-        <v>44</v>
-      </c>
-      <c r="C11" t="s">
-        <v>45</v>
-      </c>
-      <c r="D11">
-        <v>4</v>
-      </c>
-      <c r="E11">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>192</v>
-      </c>
-      <c r="B12" t="s">
-        <v>46</v>
-      </c>
-      <c r="C12" t="s">
-        <v>47</v>
-      </c>
-      <c r="D12">
-        <v>3</v>
-      </c>
-      <c r="E12">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>192</v>
-      </c>
-      <c r="B13" t="s">
-        <v>48</v>
-      </c>
-      <c r="C13" t="s">
-        <v>49</v>
-      </c>
-      <c r="D13">
-        <v>4</v>
-      </c>
-      <c r="E13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>192</v>
-      </c>
-      <c r="B14" t="s">
-        <v>50</v>
-      </c>
-      <c r="C14" t="s">
-        <v>51</v>
-      </c>
-      <c r="D14">
-        <v>4</v>
-      </c>
-      <c r="E14">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>192</v>
-      </c>
-      <c r="B15" t="s">
-        <v>52</v>
-      </c>
-      <c r="C15" t="s">
-        <v>53</v>
-      </c>
-      <c r="D15">
-        <v>4</v>
-      </c>
-      <c r="E15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>193</v>
-      </c>
-      <c r="B16" t="s">
-        <v>54</v>
-      </c>
-      <c r="C16" t="s">
-        <v>55</v>
-      </c>
-      <c r="D16">
-        <v>4</v>
-      </c>
-      <c r="E16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>193</v>
-      </c>
-      <c r="B17" t="s">
-        <v>56</v>
-      </c>
-      <c r="C17" t="s">
-        <v>57</v>
-      </c>
-      <c r="D17">
-        <v>5</v>
-      </c>
-      <c r="E17">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>193</v>
-      </c>
-      <c r="B18" t="s">
-        <v>58</v>
-      </c>
-      <c r="C18" t="s">
-        <v>59</v>
-      </c>
-      <c r="D18">
-        <v>5</v>
-      </c>
-      <c r="E18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>193</v>
-      </c>
-      <c r="B19" t="s">
-        <v>60</v>
-      </c>
-      <c r="C19" t="s">
-        <v>61</v>
-      </c>
-      <c r="D19">
-        <v>4</v>
-      </c>
-      <c r="E19">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>193</v>
-      </c>
-      <c r="B20" t="s">
-        <v>62</v>
-      </c>
-      <c r="C20" t="s">
-        <v>63</v>
-      </c>
-      <c r="D20">
-        <v>3</v>
-      </c>
-      <c r="E20">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>193</v>
-      </c>
-      <c r="B21" t="s">
-        <v>64</v>
-      </c>
-      <c r="C21" t="s">
-        <v>65</v>
-      </c>
-      <c r="D21">
-        <v>4</v>
-      </c>
-      <c r="E21">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>193</v>
-      </c>
-      <c r="B22" t="s">
-        <v>66</v>
-      </c>
-      <c r="C22" t="s">
-        <v>67</v>
-      </c>
-      <c r="D22">
-        <v>5</v>
-      </c>
-      <c r="E22">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>194</v>
-      </c>
-      <c r="B23" t="s">
-        <v>68</v>
-      </c>
-      <c r="C23" t="s">
-        <v>69</v>
-      </c>
-      <c r="D23">
-        <v>5</v>
-      </c>
-      <c r="E23">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>194</v>
-      </c>
-      <c r="B24" t="s">
-        <v>70</v>
-      </c>
-      <c r="C24" t="s">
-        <v>20</v>
-      </c>
-      <c r="D24">
-        <v>5</v>
-      </c>
-      <c r="E24">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>194</v>
-      </c>
-      <c r="B25" t="s">
-        <v>71</v>
-      </c>
-      <c r="C25" t="s">
-        <v>72</v>
-      </c>
-      <c r="D25">
-        <v>3</v>
-      </c>
-      <c r="E25">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>194</v>
-      </c>
-      <c r="B26" t="s">
-        <v>73</v>
-      </c>
-      <c r="C26" t="s">
-        <v>74</v>
-      </c>
-      <c r="D26">
-        <v>5</v>
-      </c>
-      <c r="E26">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>194</v>
-      </c>
-      <c r="B27" t="s">
-        <v>75</v>
-      </c>
-      <c r="C27" t="s">
-        <v>76</v>
-      </c>
-      <c r="D27">
-        <v>5</v>
-      </c>
-      <c r="E27">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>194</v>
-      </c>
-      <c r="B28" t="s">
-        <v>77</v>
-      </c>
-      <c r="C28" t="s">
-        <v>78</v>
-      </c>
-      <c r="D28">
-        <v>3</v>
-      </c>
-      <c r="E28">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>194</v>
-      </c>
-      <c r="B29" t="s">
-        <v>79</v>
-      </c>
-      <c r="C29" t="s">
-        <v>80</v>
-      </c>
-      <c r="D29">
-        <v>4</v>
-      </c>
-      <c r="E29">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>194</v>
-      </c>
-      <c r="B30" t="s">
-        <v>81</v>
-      </c>
-      <c r="C30" t="s">
-        <v>82</v>
-      </c>
-      <c r="D30">
-        <v>3</v>
-      </c>
-      <c r="E30">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>195</v>
-      </c>
-      <c r="B31" t="s">
-        <v>83</v>
-      </c>
-      <c r="C31" t="s">
-        <v>84</v>
-      </c>
-      <c r="D31">
-        <v>5</v>
-      </c>
-      <c r="E31">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>195</v>
-      </c>
-      <c r="B32" t="s">
-        <v>85</v>
-      </c>
-      <c r="C32" t="s">
-        <v>86</v>
-      </c>
-      <c r="D32">
-        <v>4</v>
-      </c>
-      <c r="E32">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>195</v>
-      </c>
-      <c r="B33" t="s">
-        <v>87</v>
-      </c>
-      <c r="C33" t="s">
-        <v>88</v>
-      </c>
-      <c r="D33">
-        <v>4</v>
-      </c>
-      <c r="E33">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>195</v>
-      </c>
-      <c r="B34" t="s">
-        <v>89</v>
-      </c>
-      <c r="C34" t="s">
-        <v>90</v>
-      </c>
-      <c r="D34">
-        <v>4</v>
-      </c>
-      <c r="E34">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>195</v>
-      </c>
-      <c r="B35" t="s">
-        <v>91</v>
-      </c>
-      <c r="C35" t="s">
-        <v>92</v>
-      </c>
-      <c r="D35">
-        <v>3</v>
-      </c>
-      <c r="E35">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>195</v>
-      </c>
-      <c r="B36" t="s">
-        <v>93</v>
-      </c>
-      <c r="C36" t="s">
-        <v>94</v>
-      </c>
-      <c r="D36">
-        <v>4</v>
-      </c>
-      <c r="E36">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>195</v>
-      </c>
-      <c r="B37" t="s">
-        <v>95</v>
-      </c>
-      <c r="C37" t="s">
-        <v>96</v>
-      </c>
-      <c r="D37">
-        <v>3</v>
-      </c>
-      <c r="E37">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>195</v>
-      </c>
-      <c r="B38" t="s">
-        <v>97</v>
-      </c>
-      <c r="C38" t="s">
-        <v>98</v>
-      </c>
-      <c r="D38">
-        <v>4</v>
-      </c>
-      <c r="E38">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>196</v>
-      </c>
-      <c r="B39" t="s">
-        <v>99</v>
-      </c>
-      <c r="C39" t="s">
-        <v>100</v>
-      </c>
-      <c r="D39">
-        <v>5</v>
-      </c>
-      <c r="E39">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>196</v>
-      </c>
-      <c r="B40" t="s">
-        <v>101</v>
-      </c>
-      <c r="C40" t="s">
-        <v>102</v>
-      </c>
-      <c r="D40">
-        <v>4</v>
-      </c>
-      <c r="E40">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>196</v>
-      </c>
-      <c r="B41" t="s">
-        <v>103</v>
-      </c>
-      <c r="C41" t="s">
-        <v>104</v>
-      </c>
-      <c r="D41">
-        <v>4</v>
-      </c>
-      <c r="E41">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>196</v>
-      </c>
-      <c r="B42" t="s">
-        <v>105</v>
-      </c>
-      <c r="C42" t="s">
-        <v>106</v>
-      </c>
-      <c r="D42">
-        <v>5</v>
-      </c>
-      <c r="E42">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>196</v>
-      </c>
-      <c r="B43" t="s">
-        <v>107</v>
-      </c>
-      <c r="C43" t="s">
-        <v>108</v>
-      </c>
-      <c r="D43">
-        <v>4</v>
-      </c>
-      <c r="E43">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>196</v>
-      </c>
-      <c r="B44" t="s">
-        <v>109</v>
-      </c>
-      <c r="C44" t="s">
-        <v>110</v>
-      </c>
-      <c r="D44">
-        <v>4</v>
-      </c>
-      <c r="E44">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>196</v>
-      </c>
-      <c r="B45" t="s">
-        <v>111</v>
-      </c>
-      <c r="C45" t="s">
-        <v>112</v>
-      </c>
-      <c r="D45">
-        <v>3</v>
-      </c>
-      <c r="E45">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>197</v>
-      </c>
-      <c r="B46" t="s">
-        <v>113</v>
-      </c>
-      <c r="C46" t="s">
-        <v>114</v>
-      </c>
-      <c r="D46">
-        <v>4</v>
-      </c>
-      <c r="E46">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>197</v>
-      </c>
-      <c r="B47" t="s">
-        <v>115</v>
-      </c>
-      <c r="C47" t="s">
-        <v>116</v>
-      </c>
-      <c r="D47">
-        <v>5</v>
-      </c>
-      <c r="E47">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>197</v>
-      </c>
-      <c r="B48" t="s">
-        <v>117</v>
-      </c>
-      <c r="C48" t="s">
-        <v>118</v>
-      </c>
-      <c r="D48">
-        <v>4</v>
-      </c>
-      <c r="E48">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>197</v>
-      </c>
-      <c r="B49" t="s">
-        <v>119</v>
-      </c>
-      <c r="C49" t="s">
-        <v>120</v>
-      </c>
-      <c r="D49">
-        <v>4</v>
-      </c>
-      <c r="E49">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>197</v>
-      </c>
-      <c r="B50" t="s">
-        <v>121</v>
-      </c>
-      <c r="C50" t="s">
-        <v>122</v>
-      </c>
-      <c r="D50">
-        <v>3</v>
-      </c>
-      <c r="E50">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>197</v>
-      </c>
-      <c r="B51" t="s">
-        <v>123</v>
-      </c>
-      <c r="C51" t="s">
-        <v>124</v>
-      </c>
-      <c r="D51">
-        <v>3</v>
-      </c>
-      <c r="E51">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>197</v>
-      </c>
-      <c r="B52" t="s">
-        <v>125</v>
-      </c>
-      <c r="C52" t="s">
-        <v>126</v>
-      </c>
-      <c r="D52">
-        <v>3</v>
-      </c>
-      <c r="E52">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>198</v>
-      </c>
-      <c r="B53" t="s">
-        <v>127</v>
-      </c>
-      <c r="C53" t="s">
-        <v>128</v>
-      </c>
-      <c r="D53">
-        <v>5</v>
-      </c>
-      <c r="E53">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>198</v>
-      </c>
-      <c r="B54" t="s">
-        <v>129</v>
-      </c>
-      <c r="C54" t="s">
-        <v>130</v>
-      </c>
-      <c r="D54">
-        <v>4</v>
-      </c>
-      <c r="E54">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>198</v>
-      </c>
-      <c r="B55" t="s">
-        <v>131</v>
-      </c>
-      <c r="C55" t="s">
-        <v>132</v>
-      </c>
-      <c r="D55">
-        <v>5</v>
-      </c>
-      <c r="E55">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
-        <v>198</v>
-      </c>
-      <c r="B56" t="s">
-        <v>133</v>
-      </c>
-      <c r="C56" t="s">
-        <v>134</v>
-      </c>
-      <c r="D56">
-        <v>3</v>
-      </c>
-      <c r="E56">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>198</v>
-      </c>
-      <c r="B57" t="s">
-        <v>135</v>
-      </c>
-      <c r="C57" t="s">
-        <v>136</v>
-      </c>
-      <c r="D57">
-        <v>3</v>
-      </c>
-      <c r="E57">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>198</v>
-      </c>
-      <c r="B58" t="s">
-        <v>137</v>
-      </c>
-      <c r="C58" t="s">
-        <v>138</v>
-      </c>
-      <c r="D58">
-        <v>4</v>
-      </c>
-      <c r="E58">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>198</v>
-      </c>
-      <c r="B59" t="s">
-        <v>139</v>
-      </c>
-      <c r="C59" t="s">
-        <v>140</v>
-      </c>
-      <c r="D59">
-        <v>4</v>
-      </c>
-      <c r="E59">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
-        <v>202</v>
-      </c>
-      <c r="B60" t="s">
-        <v>141</v>
-      </c>
-      <c r="C60" t="s">
-        <v>142</v>
-      </c>
-      <c r="D60">
-        <v>3</v>
-      </c>
-      <c r="E60">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>202</v>
-      </c>
-      <c r="B61" t="s">
-        <v>143</v>
-      </c>
-      <c r="C61" t="s">
-        <v>144</v>
-      </c>
-      <c r="D61">
-        <v>3</v>
-      </c>
-      <c r="E61">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>202</v>
-      </c>
-      <c r="B62" t="s">
-        <v>145</v>
-      </c>
-      <c r="C62" t="s">
-        <v>146</v>
-      </c>
-      <c r="D62">
-        <v>4</v>
-      </c>
-      <c r="E62">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A63" s="25" t="s">
-        <v>202</v>
-      </c>
-      <c r="B63" s="25" t="s">
-        <v>147</v>
-      </c>
-      <c r="C63" s="25" t="s">
-        <v>148</v>
-      </c>
-      <c r="D63" s="25">
-        <v>3</v>
-      </c>
-      <c r="E63" s="25">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
-        <v>202</v>
-      </c>
-      <c r="B64" t="s">
-        <v>149</v>
-      </c>
-      <c r="C64" t="s">
-        <v>150</v>
-      </c>
-      <c r="D64">
-        <v>3</v>
-      </c>
-      <c r="E64">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
-        <v>202</v>
-      </c>
-      <c r="B65" t="s">
-        <v>151</v>
-      </c>
-      <c r="C65" t="s">
-        <v>152</v>
-      </c>
-      <c r="D65">
-        <v>3</v>
-      </c>
-      <c r="E65">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
-        <v>201</v>
-      </c>
-      <c r="B66" t="s">
-        <v>153</v>
-      </c>
-      <c r="C66" t="s">
-        <v>154</v>
-      </c>
-      <c r="D66">
-        <v>5</v>
-      </c>
-      <c r="E66">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>201</v>
-      </c>
-      <c r="B67" t="s">
-        <v>155</v>
-      </c>
-      <c r="C67" t="s">
-        <v>156</v>
-      </c>
-      <c r="D67">
-        <v>4</v>
-      </c>
-      <c r="E67">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
-        <v>201</v>
-      </c>
-      <c r="B68" t="s">
-        <v>157</v>
-      </c>
-      <c r="C68" t="s">
-        <v>158</v>
-      </c>
-      <c r="D68">
-        <v>4</v>
-      </c>
-      <c r="E68">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>201</v>
-      </c>
-      <c r="B69" t="s">
-        <v>159</v>
-      </c>
-      <c r="C69" t="s">
-        <v>160</v>
-      </c>
-      <c r="D69">
-        <v>5</v>
-      </c>
-      <c r="E69">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>201</v>
-      </c>
-      <c r="B70" t="s">
-        <v>161</v>
-      </c>
-      <c r="C70" t="s">
-        <v>162</v>
-      </c>
-      <c r="D70">
-        <v>4</v>
-      </c>
-      <c r="E70">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
-        <v>201</v>
-      </c>
-      <c r="B71" t="s">
-        <v>163</v>
-      </c>
-      <c r="C71" t="s">
-        <v>164</v>
-      </c>
-      <c r="D71">
-        <v>4</v>
-      </c>
-      <c r="E71">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
-        <v>200</v>
-      </c>
-      <c r="B72" t="s">
-        <v>165</v>
-      </c>
-      <c r="C72" t="s">
-        <v>166</v>
-      </c>
-      <c r="D72">
-        <v>4</v>
-      </c>
-      <c r="E72">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
-        <v>200</v>
-      </c>
-      <c r="B73" t="s">
-        <v>167</v>
-      </c>
-      <c r="C73" t="s">
-        <v>168</v>
-      </c>
-      <c r="D73">
-        <v>3</v>
-      </c>
-      <c r="E73">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
-        <v>200</v>
-      </c>
-      <c r="B74" t="s">
-        <v>169</v>
-      </c>
-      <c r="C74" t="s">
-        <v>170</v>
-      </c>
-      <c r="D74">
-        <v>5</v>
-      </c>
-      <c r="E74">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
-        <v>200</v>
-      </c>
-      <c r="B75" t="s">
-        <v>171</v>
-      </c>
-      <c r="C75" t="s">
-        <v>172</v>
-      </c>
-      <c r="D75">
-        <v>3</v>
-      </c>
-      <c r="E75">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
-        <v>200</v>
-      </c>
-      <c r="B76" t="s">
-        <v>173</v>
-      </c>
-      <c r="C76" t="s">
-        <v>174</v>
-      </c>
-      <c r="D76">
-        <v>3</v>
-      </c>
-      <c r="E76">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
-        <v>200</v>
-      </c>
-      <c r="B77" t="s">
-        <v>175</v>
-      </c>
-      <c r="C77" t="s">
-        <v>176</v>
-      </c>
-      <c r="D77">
-        <v>4</v>
-      </c>
-      <c r="E77">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
-        <v>200</v>
-      </c>
-      <c r="B78" t="s">
-        <v>177</v>
-      </c>
-      <c r="C78" t="s">
-        <v>178</v>
-      </c>
-      <c r="D78">
-        <v>4</v>
-      </c>
-      <c r="E78">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A79" t="s">
-        <v>199</v>
-      </c>
-      <c r="B79" t="s">
-        <v>179</v>
-      </c>
-      <c r="C79" t="s">
-        <v>180</v>
-      </c>
-      <c r="D79">
-        <v>5</v>
-      </c>
-      <c r="E79">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A80" t="s">
-        <v>199</v>
-      </c>
-      <c r="B80" t="s">
-        <v>181</v>
-      </c>
-      <c r="C80" t="s">
-        <v>182</v>
-      </c>
-      <c r="D80">
-        <v>3</v>
-      </c>
-      <c r="E80">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A81" t="s">
-        <v>199</v>
-      </c>
-      <c r="B81" t="s">
-        <v>183</v>
-      </c>
-      <c r="C81" t="s">
-        <v>184</v>
-      </c>
-      <c r="D81">
-        <v>3</v>
-      </c>
-      <c r="E81">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
-        <v>199</v>
-      </c>
-      <c r="B82" t="s">
-        <v>185</v>
-      </c>
-      <c r="C82" t="s">
-        <v>186</v>
-      </c>
-      <c r="D82">
-        <v>3</v>
-      </c>
-      <c r="E82">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
-        <v>199</v>
-      </c>
-      <c r="B83" t="s">
-        <v>187</v>
-      </c>
-      <c r="C83" t="s">
-        <v>188</v>
-      </c>
-      <c r="D83">
-        <v>3</v>
-      </c>
-      <c r="E83">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
-        <v>199</v>
-      </c>
-      <c r="B84" t="s">
-        <v>189</v>
-      </c>
-      <c r="C84" t="s">
-        <v>190</v>
-      </c>
-      <c r="D84">
-        <v>3</v>
-      </c>
-      <c r="E84">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A7:E84" xr:uid="{B9A493EE-0271-4CD7-8525-04393AE8438C}"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60F86B49-7700-49D5-A347-A87B0CD9D1C9}">
-  <dimension ref="A1:K47"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:K48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.140625" customWidth="1"/>
@@ -3694,8 +2101,8 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="16"/>
-      <c r="B13" s="11" t="s">
-        <v>203</v>
+      <c r="B13" s="40" t="s">
+        <v>306</v>
       </c>
       <c r="C13" s="11"/>
       <c r="D13" s="11"/>
@@ -3796,7 +2203,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="34">
         <v>1</v>
       </c>
@@ -3831,7 +2238,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="34">
         <v>2</v>
       </c>
@@ -3866,7 +2273,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="34">
         <v>3</v>
       </c>
@@ -3901,7 +2308,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="34">
         <v>4</v>
       </c>
@@ -3936,7 +2343,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="34">
         <v>5</v>
       </c>
@@ -3971,7 +2378,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="34">
         <v>6</v>
       </c>
@@ -4006,7 +2413,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="34">
         <v>7</v>
       </c>
@@ -4041,7 +2448,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="34">
         <v>8</v>
       </c>
@@ -4076,7 +2483,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="34">
         <v>9</v>
       </c>
@@ -4111,7 +2518,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="34">
         <v>10</v>
       </c>
@@ -4146,7 +2553,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="34">
         <v>11</v>
       </c>
@@ -4181,7 +2588,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="34">
         <v>12</v>
       </c>
@@ -4216,7 +2623,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="34">
         <v>13</v>
       </c>
@@ -4251,7 +2658,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="35">
         <v>14</v>
       </c>
@@ -4286,7 +2693,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="34">
         <v>15</v>
       </c>
@@ -4321,7 +2728,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="34">
         <v>16</v>
       </c>
@@ -4356,7 +2763,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="34">
         <v>17</v>
       </c>
@@ -4391,7 +2798,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="34">
         <v>18</v>
       </c>
@@ -4426,7 +2833,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="34">
         <v>19</v>
       </c>
@@ -4461,7 +2868,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="34">
         <v>20</v>
       </c>
@@ -4496,7 +2903,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="34">
         <v>21</v>
       </c>
@@ -4566,7 +2973,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="34">
         <v>23</v>
       </c>
@@ -4671,7 +3078,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="34">
         <v>26</v>
       </c>
@@ -4706,7 +3113,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="34">
         <v>27</v>
       </c>
@@ -4776,8 +3183,1649 @@
         <v>5</v>
       </c>
     </row>
+    <row r="48" spans="1:11" hidden="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <autoFilter ref="B19:K48" xr:uid="{60F86B49-7700-49D5-A347-A87B0CD9D1C9}"/>
+  <autoFilter ref="B19:K48" xr:uid="{60F86B49-7700-49D5-A347-A87B0CD9D1C9}">
+    <filterColumn colId="2">
+      <colorFilter dxfId="0"/>
+    </filterColumn>
+  </autoFilter>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8B34BCC-6511-4EA4-B349-2A5DFD03ED2A}">
+  <dimension ref="A1:E18"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="35" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="8"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="10"/>
+    </row>
+    <row r="18" spans="3:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C18" s="1"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E12" xr:uid="{C8B34BCC-6511-4EA4-B349-2A5DFD03ED2A}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9A493EE-0271-4CD7-8525-04393AE8438C}">
+  <dimension ref="A1:E86"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="40.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="45" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.5703125" customWidth="1"/>
+    <col min="5" max="5" width="14.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="13" t="s">
+        <v>205</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="15"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="16" t="s">
+        <v>191</v>
+      </c>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="17"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="B3" s="11"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="17"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="39" t="s">
+        <v>305</v>
+      </c>
+      <c r="B4" s="11"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="17"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="16"/>
+      <c r="B5" s="11"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="17"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" s="11"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="11"/>
+      <c r="E6" s="17"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="19" t="s">
+        <v>203</v>
+      </c>
+      <c r="B7" s="20"/>
+      <c r="C7" s="20"/>
+      <c r="D7" s="20"/>
+      <c r="E7" s="21"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="22" t="s">
+        <v>191</v>
+      </c>
+      <c r="B9" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" s="23" t="s">
+        <v>35</v>
+      </c>
+      <c r="D9" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="E9" s="24" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>192</v>
+      </c>
+      <c r="B10" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" t="s">
+        <v>39</v>
+      </c>
+      <c r="D10">
+        <v>4</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>192</v>
+      </c>
+      <c r="B11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11">
+        <v>5</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>192</v>
+      </c>
+      <c r="B12" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" t="s">
+        <v>43</v>
+      </c>
+      <c r="D12">
+        <v>5</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>192</v>
+      </c>
+      <c r="B13" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" t="s">
+        <v>45</v>
+      </c>
+      <c r="D13">
+        <v>4</v>
+      </c>
+      <c r="E13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>192</v>
+      </c>
+      <c r="B14" t="s">
+        <v>46</v>
+      </c>
+      <c r="C14" t="s">
+        <v>47</v>
+      </c>
+      <c r="D14">
+        <v>3</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>192</v>
+      </c>
+      <c r="B15" t="s">
+        <v>48</v>
+      </c>
+      <c r="C15" t="s">
+        <v>49</v>
+      </c>
+      <c r="D15">
+        <v>4</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>192</v>
+      </c>
+      <c r="B16" t="s">
+        <v>50</v>
+      </c>
+      <c r="C16" t="s">
+        <v>51</v>
+      </c>
+      <c r="D16">
+        <v>4</v>
+      </c>
+      <c r="E16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>192</v>
+      </c>
+      <c r="B17" t="s">
+        <v>52</v>
+      </c>
+      <c r="C17" t="s">
+        <v>53</v>
+      </c>
+      <c r="D17">
+        <v>4</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>193</v>
+      </c>
+      <c r="B18" t="s">
+        <v>54</v>
+      </c>
+      <c r="C18" t="s">
+        <v>55</v>
+      </c>
+      <c r="D18">
+        <v>4</v>
+      </c>
+      <c r="E18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>193</v>
+      </c>
+      <c r="B19" t="s">
+        <v>56</v>
+      </c>
+      <c r="C19" t="s">
+        <v>57</v>
+      </c>
+      <c r="D19">
+        <v>5</v>
+      </c>
+      <c r="E19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>193</v>
+      </c>
+      <c r="B20" t="s">
+        <v>58</v>
+      </c>
+      <c r="C20" t="s">
+        <v>59</v>
+      </c>
+      <c r="D20">
+        <v>5</v>
+      </c>
+      <c r="E20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>193</v>
+      </c>
+      <c r="B21" t="s">
+        <v>60</v>
+      </c>
+      <c r="C21" t="s">
+        <v>61</v>
+      </c>
+      <c r="D21">
+        <v>4</v>
+      </c>
+      <c r="E21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>193</v>
+      </c>
+      <c r="B22" t="s">
+        <v>62</v>
+      </c>
+      <c r="C22" t="s">
+        <v>63</v>
+      </c>
+      <c r="D22">
+        <v>3</v>
+      </c>
+      <c r="E22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>193</v>
+      </c>
+      <c r="B23" t="s">
+        <v>64</v>
+      </c>
+      <c r="C23" t="s">
+        <v>65</v>
+      </c>
+      <c r="D23">
+        <v>4</v>
+      </c>
+      <c r="E23">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>193</v>
+      </c>
+      <c r="B24" t="s">
+        <v>66</v>
+      </c>
+      <c r="C24" t="s">
+        <v>67</v>
+      </c>
+      <c r="D24">
+        <v>5</v>
+      </c>
+      <c r="E24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>194</v>
+      </c>
+      <c r="B25" t="s">
+        <v>68</v>
+      </c>
+      <c r="C25" t="s">
+        <v>69</v>
+      </c>
+      <c r="D25">
+        <v>5</v>
+      </c>
+      <c r="E25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>194</v>
+      </c>
+      <c r="B26" t="s">
+        <v>70</v>
+      </c>
+      <c r="C26" t="s">
+        <v>20</v>
+      </c>
+      <c r="D26">
+        <v>5</v>
+      </c>
+      <c r="E26">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>194</v>
+      </c>
+      <c r="B27" t="s">
+        <v>71</v>
+      </c>
+      <c r="C27" t="s">
+        <v>72</v>
+      </c>
+      <c r="D27">
+        <v>3</v>
+      </c>
+      <c r="E27">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>194</v>
+      </c>
+      <c r="B28" t="s">
+        <v>73</v>
+      </c>
+      <c r="C28" t="s">
+        <v>74</v>
+      </c>
+      <c r="D28">
+        <v>5</v>
+      </c>
+      <c r="E28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>194</v>
+      </c>
+      <c r="B29" t="s">
+        <v>75</v>
+      </c>
+      <c r="C29" t="s">
+        <v>76</v>
+      </c>
+      <c r="D29">
+        <v>5</v>
+      </c>
+      <c r="E29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>194</v>
+      </c>
+      <c r="B30" t="s">
+        <v>77</v>
+      </c>
+      <c r="C30" t="s">
+        <v>78</v>
+      </c>
+      <c r="D30">
+        <v>3</v>
+      </c>
+      <c r="E30">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>194</v>
+      </c>
+      <c r="B31" t="s">
+        <v>79</v>
+      </c>
+      <c r="C31" t="s">
+        <v>80</v>
+      </c>
+      <c r="D31">
+        <v>4</v>
+      </c>
+      <c r="E31">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>194</v>
+      </c>
+      <c r="B32" t="s">
+        <v>81</v>
+      </c>
+      <c r="C32" t="s">
+        <v>82</v>
+      </c>
+      <c r="D32">
+        <v>3</v>
+      </c>
+      <c r="E32">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>195</v>
+      </c>
+      <c r="B33" t="s">
+        <v>83</v>
+      </c>
+      <c r="C33" t="s">
+        <v>84</v>
+      </c>
+      <c r="D33">
+        <v>5</v>
+      </c>
+      <c r="E33">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>195</v>
+      </c>
+      <c r="B34" t="s">
+        <v>85</v>
+      </c>
+      <c r="C34" t="s">
+        <v>86</v>
+      </c>
+      <c r="D34">
+        <v>4</v>
+      </c>
+      <c r="E34">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>195</v>
+      </c>
+      <c r="B35" t="s">
+        <v>87</v>
+      </c>
+      <c r="C35" t="s">
+        <v>88</v>
+      </c>
+      <c r="D35">
+        <v>4</v>
+      </c>
+      <c r="E35">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>195</v>
+      </c>
+      <c r="B36" t="s">
+        <v>89</v>
+      </c>
+      <c r="C36" t="s">
+        <v>90</v>
+      </c>
+      <c r="D36">
+        <v>4</v>
+      </c>
+      <c r="E36">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>195</v>
+      </c>
+      <c r="B37" t="s">
+        <v>91</v>
+      </c>
+      <c r="C37" t="s">
+        <v>92</v>
+      </c>
+      <c r="D37">
+        <v>3</v>
+      </c>
+      <c r="E37">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>195</v>
+      </c>
+      <c r="B38" t="s">
+        <v>93</v>
+      </c>
+      <c r="C38" t="s">
+        <v>94</v>
+      </c>
+      <c r="D38">
+        <v>4</v>
+      </c>
+      <c r="E38">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>195</v>
+      </c>
+      <c r="B39" t="s">
+        <v>95</v>
+      </c>
+      <c r="C39" t="s">
+        <v>96</v>
+      </c>
+      <c r="D39">
+        <v>3</v>
+      </c>
+      <c r="E39">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>195</v>
+      </c>
+      <c r="B40" t="s">
+        <v>97</v>
+      </c>
+      <c r="C40" t="s">
+        <v>98</v>
+      </c>
+      <c r="D40">
+        <v>4</v>
+      </c>
+      <c r="E40">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>196</v>
+      </c>
+      <c r="B41" t="s">
+        <v>99</v>
+      </c>
+      <c r="C41" t="s">
+        <v>100</v>
+      </c>
+      <c r="D41">
+        <v>5</v>
+      </c>
+      <c r="E41">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>196</v>
+      </c>
+      <c r="B42" t="s">
+        <v>101</v>
+      </c>
+      <c r="C42" t="s">
+        <v>102</v>
+      </c>
+      <c r="D42">
+        <v>4</v>
+      </c>
+      <c r="E42">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>196</v>
+      </c>
+      <c r="B43" t="s">
+        <v>103</v>
+      </c>
+      <c r="C43" t="s">
+        <v>104</v>
+      </c>
+      <c r="D43">
+        <v>4</v>
+      </c>
+      <c r="E43">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>196</v>
+      </c>
+      <c r="B44" t="s">
+        <v>105</v>
+      </c>
+      <c r="C44" t="s">
+        <v>106</v>
+      </c>
+      <c r="D44">
+        <v>5</v>
+      </c>
+      <c r="E44">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>196</v>
+      </c>
+      <c r="B45" t="s">
+        <v>107</v>
+      </c>
+      <c r="C45" t="s">
+        <v>108</v>
+      </c>
+      <c r="D45">
+        <v>4</v>
+      </c>
+      <c r="E45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>196</v>
+      </c>
+      <c r="B46" t="s">
+        <v>109</v>
+      </c>
+      <c r="C46" t="s">
+        <v>110</v>
+      </c>
+      <c r="D46">
+        <v>4</v>
+      </c>
+      <c r="E46">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>196</v>
+      </c>
+      <c r="B47" t="s">
+        <v>111</v>
+      </c>
+      <c r="C47" t="s">
+        <v>112</v>
+      </c>
+      <c r="D47">
+        <v>3</v>
+      </c>
+      <c r="E47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>197</v>
+      </c>
+      <c r="B48" t="s">
+        <v>113</v>
+      </c>
+      <c r="C48" t="s">
+        <v>114</v>
+      </c>
+      <c r="D48">
+        <v>4</v>
+      </c>
+      <c r="E48">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>197</v>
+      </c>
+      <c r="B49" t="s">
+        <v>115</v>
+      </c>
+      <c r="C49" t="s">
+        <v>116</v>
+      </c>
+      <c r="D49">
+        <v>5</v>
+      </c>
+      <c r="E49">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>197</v>
+      </c>
+      <c r="B50" t="s">
+        <v>117</v>
+      </c>
+      <c r="C50" t="s">
+        <v>118</v>
+      </c>
+      <c r="D50">
+        <v>4</v>
+      </c>
+      <c r="E50">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>197</v>
+      </c>
+      <c r="B51" t="s">
+        <v>119</v>
+      </c>
+      <c r="C51" t="s">
+        <v>120</v>
+      </c>
+      <c r="D51">
+        <v>4</v>
+      </c>
+      <c r="E51">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>197</v>
+      </c>
+      <c r="B52" t="s">
+        <v>121</v>
+      </c>
+      <c r="C52" t="s">
+        <v>122</v>
+      </c>
+      <c r="D52">
+        <v>3</v>
+      </c>
+      <c r="E52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>197</v>
+      </c>
+      <c r="B53" t="s">
+        <v>123</v>
+      </c>
+      <c r="C53" t="s">
+        <v>124</v>
+      </c>
+      <c r="D53">
+        <v>3</v>
+      </c>
+      <c r="E53">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>197</v>
+      </c>
+      <c r="B54" t="s">
+        <v>125</v>
+      </c>
+      <c r="C54" t="s">
+        <v>126</v>
+      </c>
+      <c r="D54">
+        <v>3</v>
+      </c>
+      <c r="E54">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>198</v>
+      </c>
+      <c r="B55" t="s">
+        <v>127</v>
+      </c>
+      <c r="C55" t="s">
+        <v>128</v>
+      </c>
+      <c r="D55">
+        <v>5</v>
+      </c>
+      <c r="E55">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>198</v>
+      </c>
+      <c r="B56" t="s">
+        <v>129</v>
+      </c>
+      <c r="C56" t="s">
+        <v>130</v>
+      </c>
+      <c r="D56">
+        <v>4</v>
+      </c>
+      <c r="E56">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>198</v>
+      </c>
+      <c r="B57" t="s">
+        <v>131</v>
+      </c>
+      <c r="C57" t="s">
+        <v>132</v>
+      </c>
+      <c r="D57">
+        <v>5</v>
+      </c>
+      <c r="E57">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>198</v>
+      </c>
+      <c r="B58" t="s">
+        <v>133</v>
+      </c>
+      <c r="C58" t="s">
+        <v>134</v>
+      </c>
+      <c r="D58">
+        <v>3</v>
+      </c>
+      <c r="E58">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>198</v>
+      </c>
+      <c r="B59" t="s">
+        <v>135</v>
+      </c>
+      <c r="C59" t="s">
+        <v>136</v>
+      </c>
+      <c r="D59">
+        <v>3</v>
+      </c>
+      <c r="E59">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>198</v>
+      </c>
+      <c r="B60" t="s">
+        <v>137</v>
+      </c>
+      <c r="C60" t="s">
+        <v>138</v>
+      </c>
+      <c r="D60">
+        <v>4</v>
+      </c>
+      <c r="E60">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>198</v>
+      </c>
+      <c r="B61" t="s">
+        <v>139</v>
+      </c>
+      <c r="C61" t="s">
+        <v>140</v>
+      </c>
+      <c r="D61">
+        <v>4</v>
+      </c>
+      <c r="E61">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>202</v>
+      </c>
+      <c r="B62" t="s">
+        <v>141</v>
+      </c>
+      <c r="C62" t="s">
+        <v>142</v>
+      </c>
+      <c r="D62">
+        <v>3</v>
+      </c>
+      <c r="E62">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>202</v>
+      </c>
+      <c r="B63" t="s">
+        <v>143</v>
+      </c>
+      <c r="C63" t="s">
+        <v>144</v>
+      </c>
+      <c r="D63">
+        <v>3</v>
+      </c>
+      <c r="E63">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>202</v>
+      </c>
+      <c r="B64" t="s">
+        <v>145</v>
+      </c>
+      <c r="C64" t="s">
+        <v>146</v>
+      </c>
+      <c r="D64">
+        <v>4</v>
+      </c>
+      <c r="E64">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A65" s="25" t="s">
+        <v>202</v>
+      </c>
+      <c r="B65" s="25" t="s">
+        <v>147</v>
+      </c>
+      <c r="C65" s="25" t="s">
+        <v>148</v>
+      </c>
+      <c r="D65" s="25">
+        <v>3</v>
+      </c>
+      <c r="E65" s="25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>202</v>
+      </c>
+      <c r="B66" t="s">
+        <v>149</v>
+      </c>
+      <c r="C66" t="s">
+        <v>150</v>
+      </c>
+      <c r="D66">
+        <v>3</v>
+      </c>
+      <c r="E66">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>202</v>
+      </c>
+      <c r="B67" t="s">
+        <v>151</v>
+      </c>
+      <c r="C67" t="s">
+        <v>152</v>
+      </c>
+      <c r="D67">
+        <v>3</v>
+      </c>
+      <c r="E67">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>201</v>
+      </c>
+      <c r="B68" t="s">
+        <v>153</v>
+      </c>
+      <c r="C68" t="s">
+        <v>154</v>
+      </c>
+      <c r="D68">
+        <v>5</v>
+      </c>
+      <c r="E68">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>201</v>
+      </c>
+      <c r="B69" t="s">
+        <v>155</v>
+      </c>
+      <c r="C69" t="s">
+        <v>156</v>
+      </c>
+      <c r="D69">
+        <v>4</v>
+      </c>
+      <c r="E69">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>201</v>
+      </c>
+      <c r="B70" t="s">
+        <v>157</v>
+      </c>
+      <c r="C70" t="s">
+        <v>158</v>
+      </c>
+      <c r="D70">
+        <v>4</v>
+      </c>
+      <c r="E70">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>201</v>
+      </c>
+      <c r="B71" t="s">
+        <v>159</v>
+      </c>
+      <c r="C71" t="s">
+        <v>160</v>
+      </c>
+      <c r="D71">
+        <v>5</v>
+      </c>
+      <c r="E71">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>201</v>
+      </c>
+      <c r="B72" t="s">
+        <v>161</v>
+      </c>
+      <c r="C72" t="s">
+        <v>162</v>
+      </c>
+      <c r="D72">
+        <v>4</v>
+      </c>
+      <c r="E72">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>201</v>
+      </c>
+      <c r="B73" t="s">
+        <v>163</v>
+      </c>
+      <c r="C73" t="s">
+        <v>164</v>
+      </c>
+      <c r="D73">
+        <v>4</v>
+      </c>
+      <c r="E73">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>200</v>
+      </c>
+      <c r="B74" t="s">
+        <v>165</v>
+      </c>
+      <c r="C74" t="s">
+        <v>166</v>
+      </c>
+      <c r="D74">
+        <v>4</v>
+      </c>
+      <c r="E74">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>200</v>
+      </c>
+      <c r="B75" t="s">
+        <v>167</v>
+      </c>
+      <c r="C75" t="s">
+        <v>168</v>
+      </c>
+      <c r="D75">
+        <v>3</v>
+      </c>
+      <c r="E75">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>200</v>
+      </c>
+      <c r="B76" t="s">
+        <v>169</v>
+      </c>
+      <c r="C76" t="s">
+        <v>170</v>
+      </c>
+      <c r="D76">
+        <v>5</v>
+      </c>
+      <c r="E76">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>200</v>
+      </c>
+      <c r="B77" t="s">
+        <v>171</v>
+      </c>
+      <c r="C77" t="s">
+        <v>172</v>
+      </c>
+      <c r="D77">
+        <v>3</v>
+      </c>
+      <c r="E77">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>200</v>
+      </c>
+      <c r="B78" t="s">
+        <v>173</v>
+      </c>
+      <c r="C78" t="s">
+        <v>174</v>
+      </c>
+      <c r="D78">
+        <v>3</v>
+      </c>
+      <c r="E78">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>200</v>
+      </c>
+      <c r="B79" t="s">
+        <v>175</v>
+      </c>
+      <c r="C79" t="s">
+        <v>176</v>
+      </c>
+      <c r="D79">
+        <v>4</v>
+      </c>
+      <c r="E79">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>200</v>
+      </c>
+      <c r="B80" t="s">
+        <v>177</v>
+      </c>
+      <c r="C80" t="s">
+        <v>178</v>
+      </c>
+      <c r="D80">
+        <v>4</v>
+      </c>
+      <c r="E80">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>199</v>
+      </c>
+      <c r="B81" t="s">
+        <v>179</v>
+      </c>
+      <c r="C81" t="s">
+        <v>180</v>
+      </c>
+      <c r="D81">
+        <v>5</v>
+      </c>
+      <c r="E81">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>199</v>
+      </c>
+      <c r="B82" t="s">
+        <v>181</v>
+      </c>
+      <c r="C82" t="s">
+        <v>182</v>
+      </c>
+      <c r="D82">
+        <v>3</v>
+      </c>
+      <c r="E82">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>199</v>
+      </c>
+      <c r="B83" t="s">
+        <v>183</v>
+      </c>
+      <c r="C83" t="s">
+        <v>184</v>
+      </c>
+      <c r="D83">
+        <v>3</v>
+      </c>
+      <c r="E83">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>199</v>
+      </c>
+      <c r="B84" t="s">
+        <v>185</v>
+      </c>
+      <c r="C84" t="s">
+        <v>186</v>
+      </c>
+      <c r="D84">
+        <v>3</v>
+      </c>
+      <c r="E84">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>199</v>
+      </c>
+      <c r="B85" t="s">
+        <v>187</v>
+      </c>
+      <c r="C85" t="s">
+        <v>188</v>
+      </c>
+      <c r="D85">
+        <v>3</v>
+      </c>
+      <c r="E85">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>199</v>
+      </c>
+      <c r="B86" t="s">
+        <v>189</v>
+      </c>
+      <c r="C86" t="s">
+        <v>190</v>
+      </c>
+      <c r="D86">
+        <v>3</v>
+      </c>
+      <c r="E86">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A9:E86" xr:uid="{B9A493EE-0271-4CD7-8525-04393AE8438C}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>